<commit_message>
feat: add dedicated standalone Med-Tech and Cyber Security Excel & PDF reports
</commit_message>
<xml_diff>
--- a/public/uploads/Nexora_Admin_Track_Report.xlsx
+++ b/public/uploads/Nexora_Admin_Track_Report.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cyber Security Track" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venue Breakdown Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Med-Tech Track" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track Summary Overview" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -62,7 +63,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -91,6 +92,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F3E8FF"/>
         <bgColor rgb="00F3E8FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00065F46"/>
+        <bgColor rgb="00065F46"/>
       </patternFill>
     </fill>
     <fill>
@@ -152,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -190,7 +197,13 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -199,10 +212,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -587,14 +600,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>NEXORA 2026 — CYBER SECURITY TRACK MASTER ROSTER (174 TEAMS)</t>
+          <t>NEXORA 2026 — CYBER SECURITY TRACK TEAM DETAILS (174 TEAMS)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Official Event Team Roster • Generated on August 22, 2026 • 07:18 PM • Total Registered Teams: 174</t>
+          <t>Official Team Details • Generated on August 22, 2026 • 07:24 PM • Total Registered Teams in Track: 174</t>
         </is>
       </c>
     </row>
@@ -678,7 +691,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -721,7 +734,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -764,7 +777,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -807,7 +820,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -850,7 +863,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -893,7 +906,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -936,7 +949,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -979,7 +992,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
+      <c r="H12" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1022,7 +1035,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1065,7 +1078,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
+      <c r="H14" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1108,7 +1121,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1151,7 +1164,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H16" s="8" t="inlineStr">
+      <c r="H16" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1194,7 +1207,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1237,7 +1250,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H18" s="8" t="inlineStr">
+      <c r="H18" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1280,7 +1293,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1323,7 +1336,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="H20" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1366,7 +1379,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1409,7 +1422,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H22" s="8" t="inlineStr">
+      <c r="H22" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1452,7 +1465,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1495,7 +1508,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H24" s="8" t="inlineStr">
+      <c r="H24" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1538,7 +1551,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="H25" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1581,7 +1594,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H26" s="8" t="inlineStr">
+      <c r="H26" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1624,7 +1637,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="H27" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1667,7 +1680,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H28" s="8" t="inlineStr">
+      <c r="H28" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1710,7 +1723,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="H29" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1753,7 +1766,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H30" s="8" t="inlineStr">
+      <c r="H30" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1796,7 +1809,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="H31" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1839,7 +1852,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H32" s="8" t="inlineStr">
+      <c r="H32" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1882,7 +1895,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr">
+      <c r="H33" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1925,7 +1938,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H34" s="8" t="inlineStr">
+      <c r="H34" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -1968,7 +1981,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr">
+      <c r="H35" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2011,7 +2024,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H36" s="8" t="inlineStr">
+      <c r="H36" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2054,7 +2067,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H37" s="4" t="inlineStr">
+      <c r="H37" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2097,7 +2110,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H38" s="8" t="inlineStr">
+      <c r="H38" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2140,7 +2153,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H39" s="4" t="inlineStr">
+      <c r="H39" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2183,7 +2196,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H40" s="8" t="inlineStr">
+      <c r="H40" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2226,7 +2239,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H41" s="4" t="inlineStr">
+      <c r="H41" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2269,7 +2282,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H42" s="8" t="inlineStr">
+      <c r="H42" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2312,7 +2325,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H43" s="4" t="inlineStr">
+      <c r="H43" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2355,7 +2368,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H44" s="8" t="inlineStr">
+      <c r="H44" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2398,7 +2411,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H45" s="4" t="inlineStr">
+      <c r="H45" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2441,7 +2454,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H46" s="8" t="inlineStr">
+      <c r="H46" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2484,7 +2497,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H47" s="4" t="inlineStr">
+      <c r="H47" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2527,7 +2540,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H48" s="8" t="inlineStr">
+      <c r="H48" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2570,7 +2583,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H49" s="4" t="inlineStr">
+      <c r="H49" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2613,7 +2626,7 @@
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="H50" s="8" t="inlineStr">
+      <c r="H50" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2656,7 +2669,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H51" s="4" t="inlineStr">
+      <c r="H51" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2699,7 +2712,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H52" s="8" t="inlineStr">
+      <c r="H52" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2742,7 +2755,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H53" s="4" t="inlineStr">
+      <c r="H53" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2785,7 +2798,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H54" s="8" t="inlineStr">
+      <c r="H54" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2828,7 +2841,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H55" s="4" t="inlineStr">
+      <c r="H55" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2871,7 +2884,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H56" s="8" t="inlineStr">
+      <c r="H56" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2914,7 +2927,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H57" s="4" t="inlineStr">
+      <c r="H57" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -2957,7 +2970,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H58" s="8" t="inlineStr">
+      <c r="H58" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3000,7 +3013,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H59" s="4" t="inlineStr">
+      <c r="H59" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3043,7 +3056,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H60" s="8" t="inlineStr">
+      <c r="H60" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3086,7 +3099,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H61" s="4" t="inlineStr">
+      <c r="H61" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3129,7 +3142,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H62" s="8" t="inlineStr">
+      <c r="H62" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3172,7 +3185,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H63" s="4" t="inlineStr">
+      <c r="H63" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3215,7 +3228,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H64" s="8" t="inlineStr">
+      <c r="H64" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3258,7 +3271,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H65" s="4" t="inlineStr">
+      <c r="H65" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3301,7 +3314,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H66" s="8" t="inlineStr">
+      <c r="H66" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3344,7 +3357,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H67" s="4" t="inlineStr">
+      <c r="H67" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3387,7 +3400,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H68" s="8" t="inlineStr">
+      <c r="H68" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3430,7 +3443,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H69" s="4" t="inlineStr">
+      <c r="H69" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3473,7 +3486,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H70" s="8" t="inlineStr">
+      <c r="H70" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3516,7 +3529,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H71" s="4" t="inlineStr">
+      <c r="H71" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3559,7 +3572,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H72" s="8" t="inlineStr">
+      <c r="H72" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3602,7 +3615,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H73" s="4" t="inlineStr">
+      <c r="H73" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3645,7 +3658,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H74" s="8" t="inlineStr">
+      <c r="H74" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3688,7 +3701,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H75" s="4" t="inlineStr">
+      <c r="H75" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3731,7 +3744,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H76" s="8" t="inlineStr">
+      <c r="H76" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3774,7 +3787,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H77" s="4" t="inlineStr">
+      <c r="H77" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3817,7 +3830,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H78" s="8" t="inlineStr">
+      <c r="H78" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3860,7 +3873,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H79" s="4" t="inlineStr">
+      <c r="H79" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3903,7 +3916,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H80" s="8" t="inlineStr">
+      <c r="H80" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3946,7 +3959,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H81" s="4" t="inlineStr">
+      <c r="H81" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -3989,7 +4002,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H82" s="8" t="inlineStr">
+      <c r="H82" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4032,7 +4045,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H83" s="4" t="inlineStr">
+      <c r="H83" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4075,7 +4088,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H84" s="8" t="inlineStr">
+      <c r="H84" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4118,7 +4131,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H85" s="4" t="inlineStr">
+      <c r="H85" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4161,7 +4174,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H86" s="8" t="inlineStr">
+      <c r="H86" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4204,7 +4217,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H87" s="4" t="inlineStr">
+      <c r="H87" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4247,7 +4260,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H88" s="8" t="inlineStr">
+      <c r="H88" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4290,7 +4303,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H89" s="4" t="inlineStr">
+      <c r="H89" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4333,7 +4346,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H90" s="8" t="inlineStr">
+      <c r="H90" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4376,7 +4389,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H91" s="4" t="inlineStr">
+      <c r="H91" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4419,7 +4432,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H92" s="8" t="inlineStr">
+      <c r="H92" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4462,7 +4475,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H93" s="4" t="inlineStr">
+      <c r="H93" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4505,7 +4518,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H94" s="8" t="inlineStr">
+      <c r="H94" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4548,7 +4561,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H95" s="4" t="inlineStr">
+      <c r="H95" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4591,7 +4604,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H96" s="8" t="inlineStr">
+      <c r="H96" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4634,7 +4647,7 @@
           <t>First Floor</t>
         </is>
       </c>
-      <c r="H97" s="4" t="inlineStr">
+      <c r="H97" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4677,7 +4690,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H98" s="8" t="inlineStr">
+      <c r="H98" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4720,7 +4733,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H99" s="4" t="inlineStr">
+      <c r="H99" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4763,7 +4776,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H100" s="8" t="inlineStr">
+      <c r="H100" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4806,7 +4819,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H101" s="4" t="inlineStr">
+      <c r="H101" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4849,7 +4862,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H102" s="8" t="inlineStr">
+      <c r="H102" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4892,7 +4905,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H103" s="4" t="inlineStr">
+      <c r="H103" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4935,7 +4948,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H104" s="8" t="inlineStr">
+      <c r="H104" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -4978,7 +4991,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H105" s="4" t="inlineStr">
+      <c r="H105" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5021,7 +5034,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H106" s="8" t="inlineStr">
+      <c r="H106" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5064,7 +5077,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H107" s="4" t="inlineStr">
+      <c r="H107" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5107,7 +5120,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H108" s="8" t="inlineStr">
+      <c r="H108" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5150,7 +5163,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H109" s="4" t="inlineStr">
+      <c r="H109" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5193,7 +5206,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H110" s="8" t="inlineStr">
+      <c r="H110" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5236,7 +5249,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H111" s="4" t="inlineStr">
+      <c r="H111" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5279,7 +5292,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H112" s="8" t="inlineStr">
+      <c r="H112" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5322,7 +5335,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H113" s="4" t="inlineStr">
+      <c r="H113" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5365,7 +5378,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H114" s="8" t="inlineStr">
+      <c r="H114" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5408,7 +5421,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H115" s="4" t="inlineStr">
+      <c r="H115" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5451,7 +5464,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H116" s="8" t="inlineStr">
+      <c r="H116" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5494,7 +5507,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H117" s="4" t="inlineStr">
+      <c r="H117" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5537,7 +5550,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H118" s="8" t="inlineStr">
+      <c r="H118" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5580,7 +5593,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H119" s="4" t="inlineStr">
+      <c r="H119" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5623,7 +5636,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H120" s="8" t="inlineStr">
+      <c r="H120" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5666,7 +5679,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H121" s="4" t="inlineStr">
+      <c r="H121" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5709,7 +5722,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H122" s="8" t="inlineStr">
+      <c r="H122" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5752,7 +5765,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H123" s="4" t="inlineStr">
+      <c r="H123" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5795,7 +5808,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H124" s="8" t="inlineStr">
+      <c r="H124" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5838,7 +5851,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H125" s="4" t="inlineStr">
+      <c r="H125" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5881,7 +5894,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H126" s="8" t="inlineStr">
+      <c r="H126" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5924,7 +5937,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H127" s="4" t="inlineStr">
+      <c r="H127" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -5967,7 +5980,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H128" s="8" t="inlineStr">
+      <c r="H128" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6010,7 +6023,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H129" s="4" t="inlineStr">
+      <c r="H129" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6053,7 +6066,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H130" s="8" t="inlineStr">
+      <c r="H130" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6096,7 +6109,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H131" s="4" t="inlineStr">
+      <c r="H131" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6139,7 +6152,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H132" s="8" t="inlineStr">
+      <c r="H132" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6182,7 +6195,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H133" s="4" t="inlineStr">
+      <c r="H133" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6225,7 +6238,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H134" s="8" t="inlineStr">
+      <c r="H134" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6268,7 +6281,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H135" s="4" t="inlineStr">
+      <c r="H135" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6311,7 +6324,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H136" s="8" t="inlineStr">
+      <c r="H136" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6354,7 +6367,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H137" s="4" t="inlineStr">
+      <c r="H137" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6397,7 +6410,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H138" s="8" t="inlineStr">
+      <c r="H138" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6440,7 +6453,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H139" s="4" t="inlineStr">
+      <c r="H139" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6483,7 +6496,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H140" s="8" t="inlineStr">
+      <c r="H140" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6526,7 +6539,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H141" s="4" t="inlineStr">
+      <c r="H141" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6569,7 +6582,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H142" s="8" t="inlineStr">
+      <c r="H142" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6612,7 +6625,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H143" s="4" t="inlineStr">
+      <c r="H143" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6655,7 +6668,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H144" s="8" t="inlineStr">
+      <c r="H144" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6698,7 +6711,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H145" s="4" t="inlineStr">
+      <c r="H145" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6741,7 +6754,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H146" s="8" t="inlineStr">
+      <c r="H146" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6784,7 +6797,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H147" s="4" t="inlineStr">
+      <c r="H147" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6827,7 +6840,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H148" s="8" t="inlineStr">
+      <c r="H148" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6870,7 +6883,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H149" s="4" t="inlineStr">
+      <c r="H149" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6913,7 +6926,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H150" s="8" t="inlineStr">
+      <c r="H150" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6956,7 +6969,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H151" s="4" t="inlineStr">
+      <c r="H151" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -6999,7 +7012,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H152" s="8" t="inlineStr">
+      <c r="H152" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7042,7 +7055,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H153" s="4" t="inlineStr">
+      <c r="H153" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7085,7 +7098,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H154" s="8" t="inlineStr">
+      <c r="H154" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7128,7 +7141,7 @@
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="H155" s="4" t="inlineStr">
+      <c r="H155" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7171,7 +7184,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H156" s="8" t="inlineStr">
+      <c r="H156" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7214,7 +7227,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H157" s="4" t="inlineStr">
+      <c r="H157" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7257,7 +7270,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H158" s="8" t="inlineStr">
+      <c r="H158" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7300,7 +7313,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H159" s="4" t="inlineStr">
+      <c r="H159" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7343,7 +7356,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H160" s="8" t="inlineStr">
+      <c r="H160" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7386,7 +7399,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H161" s="4" t="inlineStr">
+      <c r="H161" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7429,7 +7442,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H162" s="8" t="inlineStr">
+      <c r="H162" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7472,7 +7485,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H163" s="4" t="inlineStr">
+      <c r="H163" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7515,7 +7528,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H164" s="8" t="inlineStr">
+      <c r="H164" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7558,7 +7571,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H165" s="4" t="inlineStr">
+      <c r="H165" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7601,7 +7614,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H166" s="8" t="inlineStr">
+      <c r="H166" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7644,7 +7657,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H167" s="4" t="inlineStr">
+      <c r="H167" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7687,7 +7700,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H168" s="8" t="inlineStr">
+      <c r="H168" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7730,7 +7743,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H169" s="4" t="inlineStr">
+      <c r="H169" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7773,7 +7786,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H170" s="8" t="inlineStr">
+      <c r="H170" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7816,7 +7829,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H171" s="4" t="inlineStr">
+      <c r="H171" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7859,7 +7872,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H172" s="8" t="inlineStr">
+      <c r="H172" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7902,7 +7915,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H173" s="4" t="inlineStr">
+      <c r="H173" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7945,7 +7958,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H174" s="8" t="inlineStr">
+      <c r="H174" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -7988,7 +8001,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H175" s="4" t="inlineStr">
+      <c r="H175" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -8031,7 +8044,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H176" s="8" t="inlineStr">
+      <c r="H176" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -8074,7 +8087,7 @@
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="H177" s="4" t="inlineStr">
+      <c r="H177" s="7" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -8117,7 +8130,7 @@
           <t>Main Venue</t>
         </is>
       </c>
-      <c r="H178" s="8" t="inlineStr">
+      <c r="H178" s="11" t="inlineStr">
         <is>
           <t>Cyber Security</t>
         </is>
@@ -8143,196 +8156,299 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>NEXORA 2026 — CYBER SECURITY VENUE DISTRIBUTION</t>
+          <t>NEXORA 2026 — MED-TECH TRACK TEAM DETAILS (0 TEAMS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Official Team Details • Generated on August 22, 2026 • 07:24 PM • Total Registered Teams in Track: 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="10" customHeight="1"/>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>S.No</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Team ID</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Team Name</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Team Leader Name</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>Contact Phone</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>Team Size</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>Assigned Venue / Floor</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>Submission Status</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="47" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>NEXORA 2026 — MASTER TRACK &amp; VENUE SUMMARY</t>
         </is>
       </c>
     </row>
     <row r="2"/>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Venue / Location</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>ID Range</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>Track Name</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Cyber Security</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>Med-Tech</t>
+        </is>
+      </c>
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Total Teams</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>Percentage</t>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>Track Split %</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Ground Floor</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>NEX0001 - NEX0046</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
-        <is>
-          <t>Cyber Security</t>
-        </is>
-      </c>
-      <c r="D4" s="15" t="n">
+      <c r="C4" s="17" t="n">
         <v>46</v>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="D4" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="17" t="n">
+        <v>46</v>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>26.4%</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Main Venue</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>Cyber Security</t>
-        </is>
-      </c>
-      <c r="D5" s="15" t="n">
+      <c r="C5" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="D5" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>0.6%</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>First Floor</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>NEX1001 - NEX1047</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>Cyber Security</t>
-        </is>
-      </c>
-      <c r="D6" s="15" t="n">
+      <c r="C6" s="17" t="n">
         <v>47</v>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="D6" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>47</v>
+      </c>
+      <c r="F6" s="17" t="inlineStr">
         <is>
           <t>27.0%</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Second Floor</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>NEX2001 - NEX2058</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>Cyber Security</t>
-        </is>
-      </c>
-      <c r="D7" s="15" t="n">
+      <c r="C7" s="17" t="n">
         <v>58</v>
       </c>
-      <c r="E7" s="15" t="inlineStr">
+      <c r="D7" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>58</v>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>33.3%</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Online / Virtual</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>NEX3001 - NEX3023</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
-        <is>
-          <t>Cyber Security</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="n">
+      <c r="C8" s="17" t="n">
         <v>22</v>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="D8" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>22</v>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>12.6%</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>ALL VENUES</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
-        <is>
-          <t>Cyber Security</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="n">
+      <c r="C9" s="19" t="n">
         <v>174</v>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="D9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>174</v>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
@@ -8340,7 +8456,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>